<commit_message>
Project-3 : Test Cases of Microsoft Blank Document
</commit_message>
<xml_diff>
--- a/Project-3/MS_blank_test_Cases.xlsx
+++ b/Project-3/MS_blank_test_Cases.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://interbizconsult-my.sharepoint.com/personal/anjali_khute_interbizconsulting_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\source\repos\Anjali_khute_100426\Project-3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1153" documentId="8_{D09BA538-1F61-4620-B778-50375BFF0DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45466FC5-77EE-4F77-94B1-0A5FBE059F69}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Blank Docs" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,11 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="272">
-  <si>
-    <t>Project - 3 : Test case of Microsoft Blank Document
-Name : Anjali Khute</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="288">
   <si>
     <t>Module</t>
   </si>
@@ -123,9 +118,6 @@
   </si>
   <si>
     <t>Blank document opened</t>
-  </si>
-  <si>
-    <t>1. Observe cursor position</t>
   </si>
   <si>
     <t>Cursor is at top-left of page</t>
@@ -467,9 +459,6 @@
     <t>Verify font preview updates</t>
   </si>
   <si>
-    <t>1. Change font settings</t>
-  </si>
-  <si>
     <t>Preview updates correctly</t>
   </si>
   <si>
@@ -551,9 +540,6 @@
     <t>Verify paragraph preview</t>
   </si>
   <si>
-    <t>1. Modify settings</t>
-  </si>
-  <si>
     <t>Preview reflects changes</t>
   </si>
   <si>
@@ -567,9 +553,6 @@
   </si>
   <si>
     <t>Incorrect word typed</t>
-  </si>
-  <si>
-    <t>1. Right-click word</t>
   </si>
   <si>
     <t>Suggestions displayed</t>
@@ -684,9 +667,6 @@
     <t>No text selected</t>
   </si>
   <si>
-    <t>1. Right-click</t>
-  </si>
-  <si>
     <t>Cut/Copy disabled</t>
   </si>
   <si>
@@ -696,9 +676,6 @@
     <t>Verify Cut</t>
   </si>
   <si>
-    <t>1. Press Ctrl+X</t>
-  </si>
-  <si>
     <t>Text removed &amp; copied</t>
   </si>
   <si>
@@ -708,9 +685,6 @@
     <t>Verify Copy</t>
   </si>
   <si>
-    <t>1. Press Ctrl+C</t>
-  </si>
-  <si>
     <t>Text copied</t>
   </si>
   <si>
@@ -723,9 +697,6 @@
     <t>Content copied</t>
   </si>
   <si>
-    <t>1. Paste → Keep Source</t>
-  </si>
-  <si>
     <t>Text pasted</t>
   </si>
   <si>
@@ -735,16 +706,10 @@
     <t>Verify Paste (Merge Formatting)</t>
   </si>
   <si>
-    <t>1. Paste → Merge</t>
-  </si>
-  <si>
     <t>TC043</t>
   </si>
   <si>
     <t>Verify Paste (Text Only)</t>
-  </si>
-  <si>
-    <t>1. Paste → Text Only</t>
   </si>
   <si>
     <t>Plain text pasted</t>
@@ -779,9 +744,6 @@
     <t>Document open</t>
   </si>
   <si>
-    <t>1. Adjust zoom slider</t>
-  </si>
-  <si>
     <t>Zoom level changes</t>
   </si>
   <si>
@@ -794,9 +756,6 @@
     <t>Verify word count updates</t>
   </si>
   <si>
-    <t>1. Observe word count</t>
-  </si>
-  <si>
     <t>Count updates correctly</t>
   </si>
   <si>
@@ -807,9 +766,6 @@
   </si>
   <si>
     <t>Verify save default format</t>
-  </si>
-  <si>
-    <t>1. Save file</t>
   </si>
   <si>
     <t>Saved as .docx</t>
@@ -843,9 +799,6 @@
     <t>Unsaved document</t>
   </si>
   <si>
-    <t>1. Close document</t>
-  </si>
-  <si>
     <t>Save warning displayed</t>
   </si>
   <si>
@@ -861,9 +814,6 @@
     <t>System ready</t>
   </si>
   <si>
-    <t>1. Open blank doc</t>
-  </si>
-  <si>
     <t>Loads ≤ 3 seconds</t>
   </si>
   <si>
@@ -892,13 +842,119 @@
   </si>
   <si>
     <t>Ctrl+B/I/U/C/X/V/Z/Y/S</t>
+  </si>
+  <si>
+    <t>Header / Footer</t>
+  </si>
+  <si>
+    <t>Verify user can add header &amp; footer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Header &amp; Footer displayed </t>
+  </si>
+  <si>
+    <t>Double-click the header section</t>
+  </si>
+  <si>
+    <t>Change font settings</t>
+  </si>
+  <si>
+    <t>Close document</t>
+  </si>
+  <si>
+    <t>Open blank doc</t>
+  </si>
+  <si>
+    <t>Save file</t>
+  </si>
+  <si>
+    <t>Observe word count</t>
+  </si>
+  <si>
+    <t>Adjust zoom slider</t>
+  </si>
+  <si>
+    <t>Paste → Text Only</t>
+  </si>
+  <si>
+    <t>Paste → Merge</t>
+  </si>
+  <si>
+    <t>Right-click</t>
+  </si>
+  <si>
+    <t>Press Ctrl+X</t>
+  </si>
+  <si>
+    <t>Press Ctrl+C</t>
+  </si>
+  <si>
+    <t>Paste → Keep Source</t>
+  </si>
+  <si>
+    <t>Right-click word</t>
+  </si>
+  <si>
+    <t>Modify settings</t>
+  </si>
+  <si>
+    <t>Observe cursor position</t>
+  </si>
+  <si>
+    <t>TC053</t>
+  </si>
+  <si>
+    <t>TC055</t>
+  </si>
+  <si>
+    <t>Font – Advanced</t>
+  </si>
+  <si>
+    <t>Verify advanced font settings can be applied</t>
+  </si>
+  <si>
+    <t>Advanced font settings applied correctly to selected text</t>
+  </si>
+  <si>
+    <t>1. Select text
+2. Right-click → Font
+3. Open Advanced tab
+4. Change character spacing / scale
+5. Enable kerning (if available)
+6. Click OK</t>
+  </si>
+  <si>
+    <t>Paragraph – Line &amp; Page Breaks</t>
+  </si>
+  <si>
+    <t>Verify paragraph line &amp; page break settings</t>
+  </si>
+  <si>
+    <t>Multiple paragraphs exist</t>
+  </si>
+  <si>
+    <t>Paragraph behavior changes according to selected settings</t>
+  </si>
+  <si>
+    <t>1. Select paragraph
+2. Right-click → Paragraph
+3. Open Line and Page Breaks tab
+4. Enable options (Widow/Orphan, Keep with next, Page break before)
+5. Click OK</t>
+  </si>
+  <si>
+    <t>TC054</t>
+  </si>
+  <si>
+    <t>Project - 3 : Test Cases of Microsoft Blank Document
+Name : Anjali Khute</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1068,7 +1124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1141,6 +1197,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1449,9 +1508,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ACC011B-5E54-49C4-9B98-AC61B432301C}">
-  <dimension ref="A1:J56"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J59"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" style="1" customWidth="1"/>
@@ -1465,9 +1524,9 @@
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="38.25" customHeight="1">
+    <row r="1" spans="1:10" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>0</v>
+        <v>287</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -1479,7 +1538,7 @@
       <c r="I1" s="17"/>
       <c r="J1" s="18"/>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="19"/>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -1491,1200 +1550,1284 @@
       <c r="I2" s="20"/>
       <c r="J2" s="21"/>
     </row>
-    <row r="3" spans="1:10" s="2" customFormat="1" ht="24" customHeight="1">
+    <row r="3" spans="1:10" s="2" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="7" t="s">
+    </row>
+    <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="30" customHeight="1">
-      <c r="A4" s="22" t="s">
+      <c r="B4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="C4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="D4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="E4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>17</v>
-      </c>
       <c r="J4" s="3"/>
     </row>
-    <row r="5" spans="1:10" ht="30.75">
+    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="23"/>
       <c r="B5" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="D5" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="E5" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="F5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="12" t="s">
-        <v>23</v>
-      </c>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:10" ht="20.25" customHeight="1">
+    <row r="6" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="23"/>
       <c r="B6" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="D6" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="E6" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="F6" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="G6" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>29</v>
-      </c>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:10" ht="45.75">
+    <row r="7" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="23"/>
       <c r="B7" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="E7" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="G7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>34</v>
-      </c>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:10" ht="30" customHeight="1">
+    <row r="8" spans="1:10" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="23"/>
       <c r="B8" s="11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>36</v>
+        <v>256</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>37</v>
+        <v>257</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>38</v>
+        <v>259</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>39</v>
+        <v>258</v>
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:10" ht="33.75" customHeight="1">
+    <row r="9" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="23"/>
       <c r="B9" s="11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:10" ht="33.75" customHeight="1">
+    <row r="10" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="23"/>
       <c r="B10" s="11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E10" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>50</v>
-      </c>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:10" ht="23.25" customHeight="1">
+    <row r="11" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="23"/>
       <c r="B11" s="11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>55</v>
+        <v>41</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="J11" s="3"/>
     </row>
-    <row r="12" spans="1:10" ht="23.25" customHeight="1">
+    <row r="12" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="23"/>
       <c r="B12" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="J12" s="3"/>
     </row>
-    <row r="13" spans="1:10" ht="31.5" customHeight="1">
+    <row r="13" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="23"/>
       <c r="B13" s="11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>67</v>
+        <v>58</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>59</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="J13" s="3"/>
     </row>
-    <row r="14" spans="1:10" ht="36.75" customHeight="1">
+    <row r="14" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="23"/>
       <c r="B14" s="11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10" ht="34.5" customHeight="1">
+    <row r="15" spans="1:10" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="23"/>
       <c r="B15" s="11" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="E15" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G15" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>79</v>
-      </c>
       <c r="J15" s="3"/>
     </row>
-    <row r="16" spans="1:10" ht="23.25" customHeight="1">
+    <row r="16" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="23"/>
       <c r="B16" s="11" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C16" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>83</v>
-      </c>
       <c r="G16" s="12" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:10" ht="23.25" customHeight="1">
+    <row r="17" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="23"/>
       <c r="B17" s="11" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="J17" s="3"/>
     </row>
-    <row r="18" spans="1:10" ht="47.25" customHeight="1">
+    <row r="18" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="23"/>
       <c r="B18" s="11" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="E18" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="G18" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>94</v>
-      </c>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:10" ht="35.25" customHeight="1">
+    <row r="19" spans="1:10" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="23"/>
       <c r="B19" s="11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:10" ht="48.75" customHeight="1">
+    <row r="20" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="23"/>
       <c r="B20" s="11" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="J20" s="3"/>
     </row>
-    <row r="21" spans="1:10" ht="35.25" customHeight="1">
+    <row r="21" spans="1:10" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="23"/>
       <c r="B21" s="11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="J21" s="3"/>
     </row>
-    <row r="22" spans="1:10" ht="48" customHeight="1">
+    <row r="22" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="23"/>
       <c r="B22" s="11" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>111</v>
+        <v>9</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>114</v>
+        <v>70</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>106</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10" ht="35.25" customHeight="1">
+    <row r="23" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="23"/>
       <c r="B23" s="11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C23" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="E23" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="D23" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>119</v>
+      <c r="F23" s="13" t="s">
+        <v>112</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="J23" s="3"/>
     </row>
-    <row r="24" spans="1:10" ht="35.25" customHeight="1">
+    <row r="24" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="23"/>
       <c r="B24" s="11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="E24" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G24" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>124</v>
-      </c>
       <c r="J24" s="3"/>
     </row>
-    <row r="25" spans="1:10" ht="35.25" customHeight="1">
+    <row r="25" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="23"/>
       <c r="B25" s="11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="J25" s="3"/>
     </row>
-    <row r="26" spans="1:10" ht="48.75" customHeight="1">
+    <row r="26" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="23"/>
       <c r="B26" s="11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:10" ht="29.25" customHeight="1">
+    <row r="27" spans="1:10" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="23"/>
       <c r="B27" s="11" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="F27" s="12" t="s">
-        <v>135</v>
+        <v>116</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>129</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="J27" s="3"/>
     </row>
-    <row r="28" spans="1:10" ht="48.75" customHeight="1">
+    <row r="28" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="23"/>
       <c r="B28" s="11" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="F28" s="13" t="s">
-        <v>140</v>
+        <v>116</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>260</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:10" ht="35.25" customHeight="1">
+    <row r="29" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="23"/>
       <c r="B29" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="E29" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="G29" s="12" t="s">
-        <v>146</v>
+        <v>139</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F29" s="25" t="s">
+        <v>280</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>279</v>
       </c>
       <c r="J29" s="3"/>
     </row>
-    <row r="30" spans="1:10" ht="35.25" customHeight="1">
+    <row r="30" spans="1:10" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="23"/>
       <c r="B30" s="11" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C30" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="G30" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="D30" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="E30" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="G30" s="12" t="s">
-        <v>150</v>
-      </c>
       <c r="J30" s="3"/>
     </row>
-    <row r="31" spans="1:10" ht="35.25" customHeight="1">
+    <row r="31" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="23"/>
       <c r="B31" s="11" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="J31" s="3"/>
     </row>
-    <row r="32" spans="1:10" ht="35.25" customHeight="1">
+    <row r="32" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="23"/>
       <c r="B32" s="11" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="J32" s="3"/>
     </row>
-    <row r="33" spans="1:10" ht="35.25" customHeight="1">
+    <row r="33" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="23"/>
       <c r="B33" s="11" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="F33" s="12" t="s">
-        <v>161</v>
+        <v>141</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>150</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="J33" s="3"/>
     </row>
-    <row r="34" spans="1:10" ht="23.25" customHeight="1">
+    <row r="34" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="23"/>
       <c r="B34" s="11" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="F34" s="12" t="s">
-        <v>167</v>
+        <v>141</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>154</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>168</v>
+        <v>155</v>
       </c>
       <c r="J34" s="3"/>
     </row>
-    <row r="35" spans="1:10" ht="29.25" customHeight="1">
+    <row r="35" spans="1:10" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="23"/>
       <c r="B35" s="11" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>172</v>
+        <v>141</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>273</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="J35" s="3"/>
     </row>
-    <row r="36" spans="1:10" ht="32.25" customHeight="1">
+    <row r="36" spans="1:10" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="23"/>
       <c r="B36" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="D36" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="E36" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="G36" s="12" t="s">
-        <v>177</v>
+        <v>169</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="F36" s="25" t="s">
+        <v>285</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>284</v>
       </c>
       <c r="J36" s="3"/>
     </row>
-    <row r="37" spans="1:10" ht="31.5" customHeight="1">
+    <row r="37" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="23"/>
       <c r="B37" s="11" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>179</v>
+        <v>160</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>180</v>
+        <v>161</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>181</v>
+        <v>162</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>272</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>182</v>
+        <v>163</v>
       </c>
       <c r="J37" s="3"/>
     </row>
-    <row r="38" spans="1:10" ht="47.25" customHeight="1">
+    <row r="38" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="23"/>
       <c r="B38" s="11" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>72</v>
+        <v>166</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="J38" s="3"/>
     </row>
-    <row r="39" spans="1:10" ht="31.5" customHeight="1">
+    <row r="39" spans="1:10" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="23"/>
       <c r="B39" s="11" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>192</v>
+        <v>171</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>193</v>
+        <v>172</v>
       </c>
       <c r="J39" s="3"/>
     </row>
-    <row r="40" spans="1:10" ht="33" customHeight="1">
+    <row r="40" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="23"/>
       <c r="B40" s="11" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>195</v>
+        <v>174</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>196</v>
+        <v>175</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>191</v>
+        <v>70</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>197</v>
+        <v>176</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="J40" s="3"/>
     </row>
-    <row r="41" spans="1:10" ht="31.5" customHeight="1">
+    <row r="41" spans="1:10" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="23"/>
       <c r="B41" s="11" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>201</v>
+        <v>179</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>180</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="F41" s="12" t="s">
-        <v>203</v>
+        <v>70</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>181</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="J41" s="3"/>
     </row>
-    <row r="42" spans="1:10" ht="23.25" customHeight="1">
+    <row r="42" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="23"/>
       <c r="B42" s="11" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>200</v>
+        <v>184</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="F42" s="12" t="s">
-        <v>207</v>
+        <v>186</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>187</v>
       </c>
       <c r="G42" s="12" t="s">
-        <v>208</v>
+        <v>188</v>
       </c>
       <c r="J42" s="3"/>
     </row>
-    <row r="43" spans="1:10" ht="23.25" customHeight="1">
+    <row r="43" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="23"/>
       <c r="B43" s="11" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>210</v>
+        <v>191</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="F43" s="12" t="s">
-        <v>211</v>
+        <v>186</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>192</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>212</v>
+        <v>193</v>
       </c>
       <c r="J43" s="3"/>
     </row>
-    <row r="44" spans="1:10" ht="23.25" customHeight="1">
+    <row r="44" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="23"/>
       <c r="B44" s="11" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="D44" s="12" t="s">
-        <v>214</v>
+        <v>195</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>196</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>215</v>
+        <v>197</v>
       </c>
       <c r="F44" s="12" t="s">
-        <v>216</v>
+        <v>268</v>
       </c>
       <c r="G44" s="12" t="s">
-        <v>217</v>
+        <v>198</v>
       </c>
       <c r="J44" s="3"/>
     </row>
-    <row r="45" spans="1:10" ht="23.25" customHeight="1">
+    <row r="45" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="23"/>
       <c r="B45" s="11" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="C45" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="D45" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="D45" s="12" t="s">
-        <v>219</v>
-      </c>
       <c r="E45" s="12" t="s">
-        <v>215</v>
+        <v>85</v>
       </c>
       <c r="F45" s="12" t="s">
-        <v>220</v>
+        <v>269</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="J45" s="3"/>
     </row>
-    <row r="46" spans="1:10" ht="23.25" customHeight="1">
+    <row r="46" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="23"/>
       <c r="B46" s="11" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>222</v>
+        <v>203</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>215</v>
+        <v>85</v>
       </c>
       <c r="F46" s="12" t="s">
-        <v>223</v>
+        <v>270</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>224</v>
+        <v>204</v>
       </c>
       <c r="J46" s="3"/>
     </row>
-    <row r="47" spans="1:10" ht="47.25" customHeight="1">
+    <row r="47" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="23"/>
       <c r="B47" s="11" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>226</v>
+        <v>195</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>227</v>
+        <v>206</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>228</v>
+        <v>207</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>271</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>229</v>
+        <v>208</v>
       </c>
       <c r="J47" s="3"/>
     </row>
-    <row r="48" spans="1:10" ht="23.25" customHeight="1">
+    <row r="48" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="23"/>
       <c r="B48" s="11" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>231</v>
+        <v>195</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>233</v>
+        <v>207</v>
       </c>
       <c r="F48" s="12" t="s">
-        <v>234</v>
+        <v>267</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>235</v>
+        <v>208</v>
       </c>
       <c r="J48" s="3"/>
     </row>
-    <row r="49" spans="1:10" ht="23.25" customHeight="1">
+    <row r="49" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="23"/>
       <c r="B49" s="11" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>237</v>
+        <v>195</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>238</v>
+        <v>212</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>43</v>
+        <v>207</v>
       </c>
       <c r="F49" s="12" t="s">
-        <v>239</v>
+        <v>266</v>
       </c>
       <c r="G49" s="12" t="s">
-        <v>240</v>
+        <v>213</v>
       </c>
       <c r="J49" s="3"/>
     </row>
-    <row r="50" spans="1:10" ht="23.25" customHeight="1">
+    <row r="50" spans="1:10" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="23"/>
       <c r="B50" s="11" t="s">
-        <v>241</v>
+        <v>228</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>242</v>
+        <v>215</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>243</v>
+        <v>216</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>233</v>
-      </c>
-      <c r="F50" s="12" t="s">
-        <v>244</v>
+        <v>70</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>217</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>245</v>
+        <v>218</v>
       </c>
       <c r="J50" s="3"/>
     </row>
-    <row r="51" spans="1:10" ht="36.75" customHeight="1">
+    <row r="51" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="23"/>
       <c r="B51" s="11" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>247</v>
+        <v>220</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>248</v>
+        <v>221</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>233</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>249</v>
+        <v>222</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>265</v>
       </c>
       <c r="G51" s="12" t="s">
-        <v>250</v>
+        <v>223</v>
       </c>
       <c r="J51" s="3"/>
     </row>
-    <row r="52" spans="1:10" ht="23.25" customHeight="1">
+    <row r="52" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="23"/>
       <c r="B52" s="11" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>252</v>
+        <v>225</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>253</v>
+        <v>226</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>254</v>
+        <v>41</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>256</v>
+        <v>227</v>
       </c>
       <c r="J52" s="3"/>
     </row>
-    <row r="53" spans="1:10" ht="23.25" customHeight="1">
+    <row r="53" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="23"/>
       <c r="B53" s="11" t="s">
-        <v>257</v>
+        <v>242</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>258</v>
+        <v>229</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>259</v>
+        <v>230</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>260</v>
+        <v>222</v>
       </c>
       <c r="F53" s="12" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="G53" s="12" t="s">
-        <v>262</v>
+        <v>231</v>
       </c>
       <c r="J53" s="3"/>
     </row>
-    <row r="54" spans="1:10" ht="23.25" customHeight="1">
+    <row r="54" spans="1:10" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="23"/>
       <c r="B54" s="11" t="s">
-        <v>263</v>
+        <v>247</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>264</v>
+        <v>233</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>265</v>
+        <v>234</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>266</v>
-      </c>
-      <c r="F54" s="12" t="s">
-        <v>267</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>268</v>
+        <v>222</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="G54" s="12" t="s">
+        <v>236</v>
       </c>
       <c r="J54" s="3"/>
     </row>
-    <row r="55" spans="1:10" ht="21" customHeight="1">
-      <c r="A55" s="24"/>
-      <c r="B55" s="14" t="s">
-        <v>269</v>
-      </c>
-      <c r="C55" s="15" t="s">
-        <v>264</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="E55" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="F55" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="G55" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="5"/>
-    </row>
-    <row r="56" spans="1:10" ht="21" customHeight="1">
-      <c r="A56" s="9"/>
+    <row r="55" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="23"/>
+      <c r="B55" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="D55" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="F55" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="G55" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="J55" s="3"/>
+    </row>
+    <row r="56" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="23"/>
+      <c r="B56" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="E56" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="F56" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="G56" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="J56" s="3"/>
+    </row>
+    <row r="57" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="23"/>
+      <c r="B57" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="F57" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="J57" s="3"/>
+    </row>
+    <row r="58" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="24"/>
+      <c r="B58" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="5"/>
+    </row>
+    <row r="59" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A4:A55"/>
+    <mergeCell ref="A4:A58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="916bbca2-194b-49aa-86f4-8501db4dcebd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010052C21E36BBF3F44D911BA1D7F17F2A94" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a7ba8cc3de402395cf516b8f3be9c771">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="916bbca2-194b-49aa-86f4-8501db4dcebd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a6bc74132e37e06a15fc09dac2772e48" ns3:_="">
     <xsd:import namespace="916bbca2-194b-49aa-86f4-8501db4dcebd"/>
@@ -2860,31 +3003,38 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="916bbca2-194b-49aa-86f4-8501db4dcebd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4E2D055-6AEB-4047-BA86-B591862A811A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A06E39D-EDE0-47C4-907F-17047601623D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="916bbca2-194b-49aa-86f4-8501db4dcebd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A9E30DC-D8A8-4784-BA9B-E99801D8835B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A9E30DC-D8A8-4784-BA9B-E99801D8835B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A06E39D-EDE0-47C4-907F-17047601623D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4E2D055-6AEB-4047-BA86-B591862A811A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="916bbca2-194b-49aa-86f4-8501db4dcebd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>